<commit_message>
Trying again to fix bordeer and missing date
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -419,7 +419,7 @@
     <col min="3" max="3" width="10" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="1" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -437,7 +437,9 @@
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3"/>
+      <c r="C2" s="3">
+        <v>44403.871640474536</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="1" gridLines="1"/>

</xml_diff>

<commit_message>
moved to streaming system for memory efficiency
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -4,28 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Summary" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Data" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="Summary" state="visible" r:id="rId3"/>
+    <sheet sheetId="2" name="Data" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Id</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>D.O.B.</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -55,9 +38,18 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0000FF"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
@@ -67,11 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -411,7 +404,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
@@ -420,29 +412,28 @@
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
+      <c r="A1" s="1" t="str">
+        <v>Id</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>Name</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>D.O.B.</v>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>24</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
+      <c r="B2" s="4" t="str">
+        <v>Test</v>
       </c>
       <c r="C2" s="3">
-        <v>44403.88447167824</v>
+        <v>44403.92390743055</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -450,10 +441,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData/>
-  <printOptions headings="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Trying fill and putting border in column style
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -30,20 +30,36 @@
       <name val="Comic Sans"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF00FF00"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -59,12 +75,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,8 +446,8 @@
       <c r="B2" s="4" t="str">
         <v>Test</v>
       </c>
-      <c r="C2" s="3">
-        <v>44403.92390743055</v>
+      <c r="C2" s="5">
+        <v>44404.602394050926</v>
       </c>
     </row>
   </sheetData>

</xml_diff>